<commit_message>
update the UI and fix bug in /stores
</commit_message>
<xml_diff>
--- a/Store_KFC.xlsx
+++ b/Store_KFC.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kfc_recruitment_website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A12FC0E5-347D-4D25-9CB8-2D14E5B39212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{267850F6-1F3E-43D5-A12F-8DE453574440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{508703D9-26F2-4AB2-B656-A2FE4389363B}"/>
   </bookViews>
@@ -11742,213 +11742,213 @@
         <v>23</v>
       </c>
     </row>
-    <row r="250" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A250" t="s">
+    <row r="250" spans="1:11" ht="18" x14ac:dyDescent="0.4">
+      <c r="A250" s="1" t="s">
         <v>845</v>
       </c>
-      <c r="B250" t="s">
+      <c r="B250" s="1" t="s">
         <v>846</v>
       </c>
-      <c r="C250" t="s">
+      <c r="C250" s="1" t="s">
         <v>847</v>
       </c>
-      <c r="D250" t="s">
+      <c r="D250" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E250" t="s">
+      <c r="E250" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F250" t="s">
+      <c r="F250" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G250" t="s">
+      <c r="G250" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H250" t="s">
+      <c r="H250" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I250">
         <v>1</v>
       </c>
-      <c r="J250" t="s">
+      <c r="J250" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K250" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="251" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A251" t="s">
+      <c r="K250" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="251" spans="1:11" ht="18" x14ac:dyDescent="0.4">
+      <c r="A251" s="1" t="s">
         <v>848</v>
       </c>
-      <c r="B251" t="s">
+      <c r="B251" s="1" t="s">
         <v>849</v>
       </c>
-      <c r="C251" t="s">
+      <c r="C251" s="1" t="s">
         <v>850</v>
       </c>
-      <c r="D251" t="s">
+      <c r="D251" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E251" t="s">
+      <c r="E251" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F251" t="s">
-        <v>29</v>
-      </c>
-      <c r="G251" t="s">
-        <v>16</v>
-      </c>
-      <c r="H251" t="s">
+      <c r="F251" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G251" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H251" s="1" t="s">
         <v>16</v>
       </c>
       <c r="I251">
         <v>1</v>
       </c>
-      <c r="J251" t="s">
+      <c r="J251" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K251" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="252" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A252" t="s">
+      <c r="K251" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="252" spans="1:11" ht="18" x14ac:dyDescent="0.4">
+      <c r="A252" s="1" t="s">
         <v>851</v>
       </c>
-      <c r="B252" t="s">
+      <c r="B252" s="1" t="s">
         <v>852</v>
       </c>
-      <c r="C252" t="s">
+      <c r="C252" s="1" t="s">
         <v>853</v>
       </c>
-      <c r="D252" t="s">
+      <c r="D252" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="E252" t="s">
+      <c r="E252" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F252" t="s">
-        <v>29</v>
-      </c>
-      <c r="G252" t="s">
-        <v>16</v>
-      </c>
-      <c r="H252" t="s">
+      <c r="F252" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G252" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H252" s="1" t="s">
         <v>16</v>
       </c>
       <c r="I252">
         <v>1</v>
       </c>
-      <c r="J252" t="s">
+      <c r="J252" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="K252" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="253" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A253" t="s">
+      <c r="K252" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="253" spans="1:11" ht="18" x14ac:dyDescent="0.4">
+      <c r="A253" s="1" t="s">
         <v>854</v>
       </c>
-      <c r="B253" t="s">
+      <c r="B253" s="1" t="s">
         <v>855</v>
       </c>
-      <c r="C253" t="s">
+      <c r="C253" s="1" t="s">
         <v>856</v>
       </c>
-      <c r="D253" t="s">
+      <c r="D253" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E253" t="s">
+      <c r="E253" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F253" t="s">
-        <v>29</v>
-      </c>
-      <c r="G253" t="s">
-        <v>16</v>
-      </c>
-      <c r="H253" t="s">
+      <c r="F253" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G253" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H253" s="1" t="s">
         <v>16</v>
       </c>
       <c r="I253">
         <v>1</v>
       </c>
-      <c r="J253" t="s">
+      <c r="J253" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K253" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="254" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A254" t="s">
+      <c r="K253" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="254" spans="1:11" ht="18" x14ac:dyDescent="0.4">
+      <c r="A254" s="1" t="s">
         <v>857</v>
       </c>
-      <c r="B254" t="s">
+      <c r="B254" s="1" t="s">
         <v>858</v>
       </c>
-      <c r="C254" t="s">
+      <c r="C254" s="1" t="s">
         <v>859</v>
       </c>
-      <c r="D254" t="s">
+      <c r="D254" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="E254" t="s">
+      <c r="E254" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F254" t="s">
-        <v>29</v>
-      </c>
-      <c r="G254" t="s">
+      <c r="F254" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G254" s="1" t="s">
         <v>860</v>
       </c>
-      <c r="H254" t="s">
+      <c r="H254" s="1" t="s">
         <v>861</v>
       </c>
       <c r="I254">
         <v>2</v>
       </c>
-      <c r="J254" t="s">
+      <c r="J254" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="K254" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="255" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A255" t="s">
+      <c r="K254" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="255" spans="1:11" ht="18" x14ac:dyDescent="0.4">
+      <c r="A255" s="1" t="s">
         <v>862</v>
       </c>
-      <c r="B255" t="s">
+      <c r="B255" s="1" t="s">
         <v>863</v>
       </c>
-      <c r="C255" t="s">
+      <c r="C255" s="1" t="s">
         <v>864</v>
       </c>
-      <c r="D255" t="s">
+      <c r="D255" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="E255" t="s">
+      <c r="E255" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F255" t="s">
-        <v>29</v>
-      </c>
-      <c r="G255" t="s">
-        <v>16</v>
-      </c>
-      <c r="H255" t="s">
+      <c r="F255" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G255" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H255" s="1" t="s">
         <v>16</v>
       </c>
       <c r="I255">
         <v>1</v>
       </c>
-      <c r="J255" t="s">
+      <c r="J255" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="K255" t="s">
+      <c r="K255" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -11961,7 +11961,7 @@
     <cfRule type="duplicateValues" priority="4"/>
     <cfRule type="duplicateValues" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B242:B249">
+  <conditionalFormatting sqref="B242:B255">
     <cfRule type="duplicateValues" priority="6"/>
     <cfRule type="duplicateValues" priority="7"/>
     <cfRule type="duplicateValues" priority="8"/>

</xml_diff>